<commit_message>
K10: blanka kort trycktes av misstag och tas bort ur spelet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/GF_Konsekvenskort.xlsx
+++ b/kortdata/GF_Konsekvenskort.xlsx
@@ -1890,7 +1890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2014,23 +2014,6 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>LÄS - SLÅ - KASTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Tomma kort</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Obs</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Två tomma kort (CSV-platshållare) trycktes med enbart malltexten (KONSEKVENSKORT · GF, rubriker och intervall utan värden).</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3943,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>30 unika (10 TID, 10 KVALITET, 10 HÅLLBARHET), 1 exemplar vardera per spel. Därtill 2 tomma kort (CSV:ns platshållarrader) som trycktes med enbart malltext — totalt 32 kort, 64 sidor i tryckfilen.</t>
+          <t>30 unika (10 TID, 10 KVALITET, 10 HÅLLBARHET), 1 exemplar vardera per spel. Därtill 2 tomma kort (CSV:ns platshållarrader) som trycktes med enbart malltext av misstag och ska tas bort ur spelet (jfr beslut K10) — totalt 32 kort, 64 sidor i tryckfilen. De tomma korten ingår inte i kortdatan.</t>
         </is>
       </c>
     </row>

</xml_diff>